<commit_message>
no one is reading this
</commit_message>
<xml_diff>
--- a/Printers.xlsx
+++ b/Printers.xlsx
@@ -474,6 +474,16 @@
           <t>bol</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EALAN</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Falan</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -489,6 +499,16 @@
           <t>bol</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EALAN</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Falan</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -504,6 +524,16 @@
           <t>bol</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>EALAN</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Falan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -519,6 +549,16 @@
           <t>bol</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EALAN</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Falan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -534,6 +574,16 @@
           <t>bol</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>iANAN</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Falan</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -549,6 +599,16 @@
           <t>bol</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>iANAN</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Falan</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -559,6 +619,11 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>iANAN</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -569,6 +634,11 @@
           <t>heavy</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>iANAN</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -584,6 +654,11 @@
           <t>t</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>iANAN</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -619,6 +694,11 @@
       <c r="A13" s="1" t="n">
         <v>0.7083333333333334</v>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Alan</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -629,6 +709,11 @@
           <t>bol</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Alan</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -639,6 +724,11 @@
           <t>bol</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Alan</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -647,6 +737,11 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>bol</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Alan</t>
         </is>
       </c>
     </row>

</xml_diff>